<commit_message>
last version where refresh button is implemented and node addition work
</commit_message>
<xml_diff>
--- a/dataset/german/Paint_1.xlsx
+++ b/dataset/german/Paint_1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="77">
   <si>
     <t xml:space="preserve">Erfassungsformular für die Pilotdatensätze in der multimodalen Datenbank "Antiziganismus und Ambivalenz in Europa (1850–1950)"</t>
   </si>
@@ -57,16 +57,8 @@
     <t xml:space="preserve">Hier können Sie ergänzende Hinweise eintragen – z. B. Titelvarianten, problematische Begriffe (mit Kommentar in eckigen Klammern), Kontexte oder technische Anmerkungen für Redaktion, andere TPs oder das Entwicklungsteam.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">Entstehungsjahr
+    <t xml:space="preserve">Entstehungsjahr
 </t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">1912</t>
@@ -133,9 +125,6 @@
     <t xml:space="preserve">Narrative / Diskurse</t>
   </si>
   <si>
-    <t xml:space="preserve">No data</t>
-  </si>
-  <si>
     <t xml:space="preserve">Maße (Höhe × Breite × Tiefe in cm) bei Objekten oder Laufzeit (Minuten) bei medialen Werken. Bei Texten Seitenanzahl angeben usw.</t>
   </si>
   <si>
@@ -181,6 +170,9 @@
   </si>
   <si>
     <t xml:space="preserve">Rezeptionsweg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No data</t>
   </si>
   <si>
     <t xml:space="preserve">Rekonstruktion der Agency von Sinti*zze und Rom*nja. In diesem Feld sollen Form(en) der Selbstermächtigung, Selbstrepräsentation oder Selbstartikulation dokumentiert werden, die im Werk sichtbar werden oder den dargestellten Personen zugeordnet werden können. Agency bezeichnet die Fähigkeit von Individuen oder Gruppen, als handelnde Subjekte aufzutreten, eigene Perspektiven sichtbar zu machen und bestehende Stereotypen oder dominante Deutungsmuster bewusst zu durchbrechen.
@@ -291,7 +283,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="d\.m\.yy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -326,17 +318,12 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
@@ -570,11 +557,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -976,12 +963,10 @@
       <c r="A12" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B12" s="7"/>
       <c r="C12" s="8"/>
       <c r="D12" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E12" s="8"/>
       <c r="F12" s="10"/>
@@ -1007,14 +992,14 @@
     </row>
     <row r="13" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" s="8"/>
       <c r="D13" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E13" s="8"/>
       <c r="F13" s="10"/>
@@ -1040,14 +1025,12 @@
     </row>
     <row r="14" customFormat="false" ht="172.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B14" s="7"/>
       <c r="C14" s="8"/>
       <c r="D14" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="10"/>
@@ -1073,14 +1056,12 @@
     </row>
     <row r="15" customFormat="false" ht="95.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B15" s="7"/>
       <c r="C15" s="8"/>
       <c r="D15" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E15" s="8"/>
       <c r="F15" s="10"/>
@@ -1106,14 +1087,12 @@
     </row>
     <row r="16" customFormat="false" ht="78.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B16" s="7"/>
       <c r="C16" s="8"/>
       <c r="D16" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E16" s="8"/>
       <c r="F16" s="10"/>
@@ -1139,14 +1118,12 @@
     </row>
     <row r="17" customFormat="false" ht="220.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B17" s="7"/>
       <c r="C17" s="8"/>
       <c r="D17" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E17" s="8"/>
       <c r="F17" s="10"/>
@@ -1172,10 +1149,10 @@
     </row>
     <row r="18" customFormat="false" ht="125.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C18" s="8"/>
       <c r="D18" s="3" t="s">
@@ -1208,7 +1185,7 @@
         <v>48</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="3" t="s">
@@ -1273,9 +1250,7 @@
       <c r="A21" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B21" s="14" t="s">
-        <v>33</v>
-      </c>
+      <c r="B21" s="14"/>
       <c r="C21" s="8"/>
       <c r="D21" s="3" t="s">
         <v>54</v>
@@ -1339,9 +1314,7 @@
       <c r="A23" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B23" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B23" s="7"/>
       <c r="C23" s="8"/>
       <c r="D23" s="3" t="s">
         <v>59</v>
@@ -1372,9 +1345,7 @@
       <c r="A24" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B24" s="7"/>
       <c r="C24" s="8"/>
       <c r="D24" s="3" t="s">
         <v>61</v>
@@ -1405,9 +1376,7 @@
       <c r="A25" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="15" t="s">
-        <v>33</v>
-      </c>
+      <c r="B25" s="15"/>
       <c r="C25" s="16"/>
       <c r="D25" s="17" t="s">
         <v>63</v>
@@ -1438,9 +1407,7 @@
       <c r="A26" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="B26" s="19" t="s">
-        <v>33</v>
-      </c>
+      <c r="B26" s="19"/>
       <c r="C26" s="20"/>
       <c r="D26" s="21" t="s">
         <v>65</v>
@@ -1471,9 +1438,7 @@
       <c r="A27" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B27" s="7"/>
       <c r="C27" s="8"/>
       <c r="D27" s="3" t="s">
         <v>67</v>
@@ -1504,9 +1469,7 @@
       <c r="A28" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="14" t="s">
-        <v>33</v>
-      </c>
+      <c r="B28" s="14"/>
       <c r="C28" s="8"/>
       <c r="D28" s="3" t="s">
         <v>69</v>
@@ -1537,9 +1500,7 @@
       <c r="A29" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="7" t="s">
-        <v>33</v>
-      </c>
+      <c r="B29" s="7"/>
       <c r="C29" s="8"/>
       <c r="D29" s="3" t="s">
         <v>71</v>
@@ -1570,9 +1531,7 @@
       <c r="A30" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="23" t="s">
-        <v>33</v>
-      </c>
+      <c r="B30" s="23"/>
       <c r="C30" s="8"/>
       <c r="D30" s="3" t="s">
         <v>73</v>

</xml_diff>